<commit_message>
New graphs + progress on LCIs
</commit_message>
<xml_diff>
--- a/results/Scenario modeling SHDB (1).xlsx
+++ b/results/Scenario modeling SHDB (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/fasc_metal_sustainability/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{D73EABFE-5DA0-4A68-BDDA-E91B083C991F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{121604F9-1382-44FE-9B53-449D1567C6E0}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{D73EABFE-5DA0-4A68-BDDA-E91B083C991F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B40FEE49-BC34-469E-80FA-F3BB2E3783A0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14192,6 +14192,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Theme_Ciraig">
   <a:themeElements>

</xml_diff>